<commit_message>
actualizar resultados finales con reportes procesados
</commit_message>
<xml_diff>
--- a/bot-ventas/resultados/consolidado_limpio.xlsx
+++ b/bot-ventas/resultados/consolidado_limpio.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G84"/>
+  <dimension ref="A1:G88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -906,12 +906,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Teclado mecanico</t>
+          <t>Teclado</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -923,11 +923,11 @@
         <v>2</v>
       </c>
       <c r="E16" t="n">
-        <v>142300</v>
+        <v>65000</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Camila Ruiz</t>
+          <t>Sofia</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -939,12 +939,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Jean clasico</t>
+          <t>Falda</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -953,14 +953,14 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>103400</v>
+        <v>52000</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Andres Gomez</t>
+          <t>Juan</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -972,12 +972,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Audifonos Bluetooth</t>
+          <t>Audifonos</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -986,31 +986,31 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E18" t="n">
-        <v>167200</v>
+        <v>38000</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Sofia Mena</t>
+          <t>Sofia</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Transferencia</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Camiseta basica</t>
+          <t>Chaqueta</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1019,31 +1019,31 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>56100</v>
+        <v>120000</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Laura Diaz</t>
+          <t>Juan</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Efectivo</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Parlante portatil</t>
+          <t>Teclado mecanico</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1052,31 +1052,31 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E20" t="n">
-        <v>98700</v>
+        <v>142300</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Felipe Torres</t>
+          <t>Camila Ruiz</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Chaqueta impermeable</t>
+          <t>Jean clasico</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1085,31 +1085,31 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E21" t="n">
-        <v>145600</v>
+        <v>103400</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Camila Ruiz</t>
+          <t>Andres Gomez</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Efectivo</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Mouse inalambrico</t>
+          <t>Audifonos Bluetooth</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1118,97 +1118,97 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>73800</v>
+        <v>167200</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Andres Gomez</t>
+          <t>Sofia Mena</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Transferencia</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Cargador USB-C</t>
+          <t>Camiseta basica</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D23" t="n">
         <v>3</v>
       </c>
       <c r="E23" t="n">
-        <v>112500</v>
+        <v>56100</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Sofia Mena</t>
+          <t>Laura Diaz</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Transferencia</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Medias deportivas</t>
+          <t>Parlante portatil</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D24" t="n">
         <v>4</v>
       </c>
       <c r="E24" t="n">
-        <v>28900</v>
+        <v>98700</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Laura Diaz</t>
+          <t>Felipe Torres</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Efectivo</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Gorra deportiva</t>
+          <t>Chaqueta impermeable</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1217,14 +1217,14 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E25" t="n">
-        <v>74300</v>
+        <v>145600</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Felipe Torres</t>
+          <t>Camila Ruiz</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1236,24 +1236,24 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Camiseta basica</t>
+          <t>Mouse inalambrico</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E26" t="n">
-        <v>55400</v>
+        <v>73800</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1262,19 +1262,19 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Efectivo</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Parlante portatil</t>
+          <t>Cargador USB-C</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1283,31 +1283,31 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E27" t="n">
-        <v>20200</v>
+        <v>112500</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Camila Ruiz</t>
+          <t>Sofia Mena</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Transferencia</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Jean clasico</t>
+          <t>Medias deportivas</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1316,27 +1316,31 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E28" t="n">
-        <v>107600</v>
+        <v>28900</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Sofia Mena</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr"/>
+          <t>Laura Diaz</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Efectivo</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Jean clasico</t>
+          <t>Gorra deportiva</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1345,47 +1349,47 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>148600</v>
+        <v>74300</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Camila Ruiz</t>
+          <t>Felipe Torres</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Teclado mecanico</t>
+          <t>Camiseta basica</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D30" t="n">
         <v>5</v>
       </c>
       <c r="E30" t="n">
-        <v>40700</v>
+        <v>55400</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Laura Diaz</t>
+          <t>Andres Gomez</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1397,90 +1401,86 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Camiseta basica</t>
+          <t>Parlante portatil</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E31" t="n">
-        <v>74200</v>
+        <v>20200</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Laura Diaz</t>
+          <t>Camila Ruiz</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Transferencia</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Audifonos Bluetooth</t>
+          <t>Jean clasico</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>175600</v>
+        <v>107600</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Felipe Torres</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>Efectivo</t>
-        </is>
-      </c>
+          <t>Sofia Mena</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Parlante portatil</t>
+          <t>Jean clasico</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E33" t="n">
-        <v>110300</v>
+        <v>148600</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -1489,60 +1489,64 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Efectivo</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Jean clasico</t>
+          <t>Teclado mecanico</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E34" t="n">
-        <v>156100</v>
+        <v>40700</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Camila Ruiz</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr"/>
+          <t>Laura Diaz</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Efectivo</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Cargador USB-C</t>
+          <t>Camiseta basica</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E35" t="n">
-        <v>41800</v>
+        <v>74200</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -1551,19 +1555,19 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Transferencia</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Cargador USB-C</t>
+          <t>Audifonos Bluetooth</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1575,28 +1579,28 @@
         <v>2</v>
       </c>
       <c r="E36" t="n">
-        <v>115500</v>
+        <v>175600</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Andres Gomez</t>
+          <t>Felipe Torres</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Mouse inalambrico</t>
+          <t>Parlante portatil</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1605,31 +1609,31 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E37" t="n">
-        <v>59500</v>
+        <v>110300</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Sofia Mena</t>
+          <t>Camila Ruiz</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Chaqueta impermeable</t>
+          <t>Jean clasico</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1638,14 +1642,14 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E38" t="n">
-        <v>150600</v>
+        <v>156100</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Laura Diaz</t>
+          <t>Camila Ruiz</t>
         </is>
       </c>
       <c r="G38" t="inlineStr"/>
@@ -1653,7 +1657,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1667,47 +1671,47 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E39" t="n">
-        <v>165700</v>
+        <v>41800</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Sofia Mena</t>
+          <t>Laura Diaz</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Transferencia</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Jean clasico</t>
+          <t>Cargador USB-C</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E40" t="n">
-        <v>80300</v>
+        <v>115500</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Felipe Torres</t>
+          <t>Andres Gomez</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -1719,12 +1723,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Cargador USB-C</t>
+          <t>Mouse inalambrico</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1733,10 +1737,10 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>137900</v>
+        <v>59500</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
@@ -1745,19 +1749,19 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Transferencia</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Medias deportivas</t>
+          <t>Chaqueta impermeable</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1766,14 +1770,14 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E42" t="n">
-        <v>74700</v>
+        <v>150600</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Andres Gomez</t>
+          <t>Laura Diaz</t>
         </is>
       </c>
       <c r="G42" t="inlineStr"/>
@@ -1781,57 +1785,61 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Camiseta basica</t>
+          <t>Cargador USB-C</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E43" t="n">
-        <v>40200</v>
+        <v>165700</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Andres Gomez</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr"/>
+          <t>Sofia Mena</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Transferencia</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Audifonos Bluetooth</t>
+          <t>Jean clasico</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E44" t="n">
-        <v>185000</v>
+        <v>80300</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Andres Gomez</t>
+          <t>Felipe Torres</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -1843,73 +1851,69 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Jean clasico</t>
+          <t>Cargador USB-C</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D45" t="n">
         <v>4</v>
       </c>
       <c r="E45" t="n">
-        <v>92300</v>
+        <v>137900</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Camila Ruiz</t>
+          <t>Sofia Mena</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Efectivo</t>
+          <t>Transferencia</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Parlante portatil</t>
+          <t>Medias deportivas</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>134500</v>
+        <v>74700</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Sofia Mena</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>Transferencia</t>
-        </is>
-      </c>
+          <t>Andres Gomez</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1923,31 +1927,27 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E47" t="n">
-        <v>48700</v>
+        <v>40200</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Laura Diaz</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>Tarjeta</t>
-        </is>
-      </c>
+          <t>Andres Gomez</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Teclado mecanico</t>
+          <t>Audifonos Bluetooth</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1956,31 +1956,31 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E48" t="n">
-        <v>156800</v>
+        <v>185000</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Felipe Torres</t>
+          <t>Andres Gomez</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Efectivo</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Chaqueta impermeable</t>
+          <t>Jean clasico</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1989,31 +1989,31 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E49" t="n">
-        <v>178900</v>
+        <v>92300</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Andres Gomez</t>
+          <t>Camila Ruiz</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Cargador USB-C</t>
+          <t>Parlante portatil</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2022,80 +2022,80 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E50" t="n">
-        <v>72400</v>
+        <v>134500</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Camila Ruiz</t>
+          <t>Sofia Mena</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Efectivo</t>
+          <t>Transferencia</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Mouse inalambrico</t>
+          <t>Camiseta basica</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E51" t="n">
-        <v>89200</v>
+        <v>48700</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Sofia Mena</t>
+          <t>Laura Diaz</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Transferencia</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Medias deportivas</t>
+          <t>Teclado mecanico</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E52" t="n">
-        <v>31500</v>
+        <v>156800</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Laura Diaz</t>
+          <t>Felipe Torres</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2107,12 +2107,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Gorra deportiva</t>
+          <t>Chaqueta impermeable</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2121,14 +2121,14 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E53" t="n">
-        <v>67800</v>
+        <v>178900</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Felipe Torres</t>
+          <t>Andres Gomez</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2140,28 +2140,28 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>05/06/2026</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Chaqueta impermeable</t>
+          <t>Cargador USB-C</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E54" t="n">
-        <v>90600</v>
+        <v>72400</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Sofia Mena</t>
+          <t>Camila Ruiz</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2173,28 +2173,28 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>05/07/2026</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Camiseta basica</t>
+          <t>Mouse inalambrico</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D55" t="n">
         <v>4</v>
       </c>
       <c r="E55" t="n">
-        <v>98500</v>
+        <v>89200</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Andres Gomez</t>
+          <t>Sofia Mena</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2206,12 +2206,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>16/06/2026</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Camiseta basica</t>
+          <t>Medias deportivas</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2220,29 +2220,31 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>6</v>
-      </c>
-      <c r="E56" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="E56" t="n">
+        <v>31500</v>
+      </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Felipe Torres</t>
+          <t>Laura Diaz</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Transferencia</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>12/07/2026</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Medias deportivas</t>
+          <t>Gorra deportiva</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2251,31 +2253,31 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E57" t="n">
-        <v>125200</v>
+        <v>67800</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Sofia Mena</t>
+          <t>Felipe Torres</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Transferencia</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>09/06/2026</t>
+          <t>05/06/2026</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Camiseta basica</t>
+          <t>Chaqueta impermeable</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2284,39 +2286,43 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E58" t="n">
-        <v>34000</v>
-      </c>
-      <c r="F58" t="inlineStr"/>
+        <v>90600</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Sofia Mena</t>
+        </is>
+      </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>19/06/2026</t>
+          <t>05/07/2026</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Cargador USB-C</t>
+          <t>Camiseta basica</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D59" t="n">
         <v>4</v>
       </c>
       <c r="E59" t="n">
-        <v>133400</v>
+        <v>98500</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
@@ -2332,59 +2338,59 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>02/07/2026</t>
+          <t>16/06/2026</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Parlante portatil</t>
+          <t>Camiseta basica</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>5</v>
-      </c>
-      <c r="E60" t="n">
-        <v>164400</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Camila Ruiz</t>
+          <t>Felipe Torres</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Efectivo</t>
+          <t>Transferencia</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>12/07/2026</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Teclado mecanico</t>
+          <t>Medias deportivas</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D61" t="n">
         <v>1</v>
       </c>
-      <c r="E61" t="inlineStr"/>
+      <c r="E61" t="n">
+        <v>125200</v>
+      </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Andres Gomez</t>
+          <t>Sofia Mena</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -2396,45 +2402,41 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>29/06/2026</t>
+          <t>09/06/2026</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Mouse inalambrico</t>
+          <t>Camiseta basica</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E62" t="n">
-        <v>107500</v>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>Camila Ruiz</t>
-        </is>
-      </c>
+        <v>34000</v>
+      </c>
+      <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Efectivo</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>05/07/2026</t>
+          <t>19/06/2026</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Mouse inalambrico</t>
+          <t>Cargador USB-C</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2443,27 +2445,31 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E63" t="n">
-        <v>152700</v>
-      </c>
-      <c r="F63" t="inlineStr"/>
+        <v>133400</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Andres Gomez</t>
+        </is>
+      </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Transferencia</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>09/06/2026</t>
+          <t>02/07/2026</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Teclado mecanico</t>
+          <t>Parlante portatil</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2472,10 +2478,10 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E64" t="n">
-        <v>65900</v>
+        <v>164400</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
@@ -2484,75 +2490,83 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Transferencia</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>14/07/2026</t>
+          <t>18/06/2026</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Jean clasico</t>
+          <t>Teclado mecanico</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Laura Diaz</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr"/>
+          <t>Andres Gomez</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Transferencia</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>10/06/2026</t>
+          <t>29/06/2026</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Medias deportivas</t>
+          <t>Mouse inalambrico</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E66" t="n">
-        <v>157700</v>
+        <v>107500</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Andres Gomez</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr"/>
+          <t>Camila Ruiz</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Efectivo</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>12/06/2026</t>
+          <t>05/07/2026</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Audifonos Bluetooth</t>
+          <t>Mouse inalambrico</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2561,16 +2575,12 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E67" t="n">
-        <v>144100</v>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>Felipe Torres</t>
-        </is>
-      </c>
+        <v>152700</v>
+      </c>
+      <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
           <t>Tarjeta</t>
@@ -2580,12 +2590,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>11/06/2026</t>
+          <t>09/06/2026</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Cargador USB-C</t>
+          <t>Teclado mecanico</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -2594,22 +2604,26 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E68" t="n">
-        <v>78100</v>
+        <v>65900</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
           <t>Camila Ruiz</t>
         </is>
       </c>
-      <c r="G68" t="inlineStr"/>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Transferencia</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>13/06/2026</t>
+          <t>14/07/2026</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2623,26 +2637,20 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>8</v>
-      </c>
-      <c r="E69" t="n">
-        <v>72700</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Andres Gomez</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>Tarjeta</t>
-        </is>
-      </c>
+          <t>Laura Diaz</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>10/06/2026</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2656,31 +2664,27 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E70" t="n">
-        <v>78000</v>
+        <v>157700</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Felipe Torres</t>
-        </is>
-      </c>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t>Transferencia</t>
-        </is>
-      </c>
+          <t>Andres Gomez</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>12/06/2026</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Parlante portatil</t>
+          <t>Audifonos Bluetooth</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -2689,146 +2693,142 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E71" t="n">
-        <v>127500</v>
+        <v>144100</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Sofia Mena</t>
+          <t>Felipe Torres</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Transferencia</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>11/06/2026</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Chaqueta impermeable</t>
+          <t>Cargador USB-C</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E72" t="n">
-        <v>86700</v>
+        <v>78100</v>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Felipe Torres</t>
-        </is>
-      </c>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>Efectivo</t>
-        </is>
-      </c>
+          <t>Camila Ruiz</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>13/06/2026</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Cargador USB-C</t>
+          <t>Jean clasico</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E73" t="n">
-        <v>98800</v>
+        <v>72700</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Camila Ruiz</t>
+          <t>Andres Gomez</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Transferencia</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Parlante portatil</t>
+          <t>Medias deportivas</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E74" t="n">
-        <v>40200</v>
+        <v>78000</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Andres Gomez</t>
+          <t>Felipe Torres</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Efectivo</t>
+          <t>Transferencia</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Medias deportivas</t>
+          <t>Parlante portatil</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E75" t="n">
-        <v>18200</v>
+        <v>127500</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Laura Diaz</t>
+          <t>Sofia Mena</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -2840,12 +2840,12 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Jean clasico</t>
+          <t>Chaqueta impermeable</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -2854,14 +2854,14 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E76" t="n">
-        <v>159900</v>
+        <v>86700</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Camila Ruiz</t>
+          <t>Felipe Torres</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -2873,45 +2873,45 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Gorra deportiva</t>
+          <t>Cargador USB-C</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D77" t="n">
         <v>3</v>
       </c>
       <c r="E77" t="n">
-        <v>36200</v>
+        <v>98800</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Felipe Torres</t>
+          <t>Camila Ruiz</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Transferencia</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Cargador USB-C</t>
+          <t>Parlante portatil</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -2920,60 +2920,64 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E78" t="n">
-        <v>174100</v>
+        <v>40200</v>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Sofia Mena</t>
+          <t>Andres Gomez</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Cargador USB-C</t>
+          <t>Medias deportivas</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E79" t="n">
-        <v>87300</v>
+        <v>18200</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Sofia Mena</t>
-        </is>
-      </c>
-      <c r="G79" t="inlineStr"/>
+          <t>Laura Diaz</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Transferencia</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Camiseta basica</t>
+          <t>Jean clasico</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -2985,7 +2989,7 @@
         <v>4</v>
       </c>
       <c r="E80" t="n">
-        <v>25600</v>
+        <v>159900</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
@@ -2994,19 +2998,19 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Medias deportivas</t>
+          <t>Gorra deportiva</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3015,14 +3019,14 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E81" t="n">
-        <v>26700</v>
+        <v>36200</v>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Camila Ruiz</t>
+          <t>Felipe Torres</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -3034,57 +3038,57 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Camiseta basica</t>
+          <t>Cargador USB-C</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E82" t="n">
-        <v>26700</v>
+        <v>174100</v>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Andres Gomez</t>
+          <t>Sofia Mena</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Transferencia</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Gorra deportiva</t>
+          <t>Cargador USB-C</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E83" t="n">
-        <v>134400</v>
+        <v>87300</v>
       </c>
       <c r="F83" t="inlineStr">
         <is>
@@ -3096,31 +3100,159 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Camiseta basica</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>4</v>
+      </c>
+      <c r="E84" t="n">
+        <v>25600</v>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Camila Ruiz</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Tarjeta</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Medias deportivas</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>1</v>
+      </c>
+      <c r="E85" t="n">
+        <v>26700</v>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Camila Ruiz</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Tarjeta</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Camiseta basica</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>6</v>
+      </c>
+      <c r="E86" t="n">
+        <v>26700</v>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Andres Gomez</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Transferencia</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Gorra deportiva</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>3</v>
+      </c>
+      <c r="E87" t="n">
+        <v>134400</v>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Sofia Mena</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr">
+      <c r="B88" t="inlineStr">
         <is>
           <t>Jean clasico</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>Ropa</t>
-        </is>
-      </c>
-      <c r="D84" t="n">
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
         <v>7</v>
       </c>
-      <c r="E84" t="n">
+      <c r="E88" t="n">
         <v>46400</v>
       </c>
-      <c r="F84" t="inlineStr">
+      <c r="F88" t="inlineStr">
         <is>
           <t>Camila Ruiz</t>
         </is>
       </c>
-      <c r="G84" t="inlineStr"/>
+      <c r="G88" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>